<commit_message>
Update full_vendor_mapping_final.xlsx with manual edits
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/mappings/full_vendor_mapping_final.xlsx
+++ b/outputs/mappings/full_vendor_mapping_final.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/anakk/Desktop/Work/Vibe coding/CW Vendor Assessment/outputs/mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5129CF0D-65C6-1141-A4B3-A2EC502594DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E191D7-A86A-594E-8EE6-5F05930886DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Vendor Mapping" sheetId="1" r:id="rId1"/>
@@ -2872,7 +2872,8 @@
     <t>Support</t>
   </si>
   <si>
-    <t>prompts.md</t>
+    <t>prompts.md
+https://drive.google.com/file/d/1pev5JC1ZkmhwaIVC8EadzWxjfggm_vb8/view?usp=sharing</t>
   </si>
 </sst>
 </file>
@@ -3363,12 +3364,12 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13790,10 +13791,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="48" t="s">
         <v>910</v>
       </c>
-      <c r="B1" s="47"/>
+      <c r="B1" s="49"/>
     </row>
     <row r="2" spans="1:2" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="43" t="s">
@@ -13856,7 +13857,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="48" t="s">
         <v>920</v>
       </c>
     </row>
@@ -13883,67 +13884,67 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="46" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" s="49" t="s">
+      <c r="A2" s="47" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" s="49" t="s">
+      <c r="A3" s="47" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="47" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="47" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="49" t="s">
+      <c r="A6" s="47" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="49" t="s">
+      <c r="A7" s="47" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="47" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A9" s="49" t="s">
+      <c r="A9" s="47" t="s">
         <v>301</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" s="49" t="s">
+      <c r="A10" s="47" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" s="49" t="s">
+      <c r="A11" s="47" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" s="49" t="s">
+      <c r="A12" s="47" t="s">
         <v>922</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" s="49" t="s">
+      <c r="A13" s="47" t="s">
         <v>21</v>
       </c>
     </row>

</xml_diff>